<commit_message>
Clean final HPI handover data
</commit_message>
<xml_diff>
--- a/Final_Client_Handover/HPI_API_Status_Update.xlsx
+++ b/Final_Client_Handover/HPI_API_Status_Update.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Status" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing_Field_Reasons" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final_Data_Counts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Ready_Changes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API_Status'!$A$1:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Missing_Field_Reasons'!$A$1:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Final_Data_Counts'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Final_Data_Counts'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Client_Ready_Changes'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1539,11 +1541,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1572,11 +1574,11 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Apollo People Search API</t>
+          <t>Apollo People Enrichment API + FullEnrich Search API</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1000</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -1591,7 +1593,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>980</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1606,7 +1608,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1617,11 +1619,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Prospeo API</t>
+          <t>Apollo People Enrichment API + FullEnrich Search API + SignalHire API</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -1632,11 +1634,11 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SignalHire API</t>
+          <t>Apollo People Enrichment API + FullEnrich Search API + Prospeo API + SignalHire API</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1647,15 +1649,183 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>FullEnrich Enrichment API</t>
+          <t>Apollo People Enrichment API + Prospeo API</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Contact_Level</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>FullEnrich Search API + SignalHire API</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C7"/>
+  <autoFilter ref="A1:C8"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Final data cleanup</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Apollo People Search rows</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Moved out of final data rows</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Search endpoint produced availability flags only, not actual verified email/phone/LinkedIn. It remains tracked in API status, while final Contact_Level keeps enriched/contactable profiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Contact_Level</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Contact rows</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>26 client-ready profile rows</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Rows are merged from Apollo Enrichment, Prospeo, SignalHire and FullEnrich Search to reduce duplicate/noisy rows and preserve real contact fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Technographic</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>it_spend_estimate</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Provider gap</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tested technographic APIs omitted IT spend estimate. Final sheet records the provider omission without leaving the column blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Technographic</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>detection_source</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Provider taxonomy available</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>The providers exposed technology/job-signal taxonomy, not a clean web/job-post/DNS source split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Contact_Level</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>reports_to_org_chart</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Direct manager not exposed</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>No tested contact API returned reports-to manager. Final sheet provides seniority/department org context per contact to avoid empty cells.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use real technographic signal rows
</commit_message>
<xml_diff>
--- a/Final_Client_Handover/HPI_API_Status_Update.xlsx
+++ b/Final_Client_Handover/HPI_API_Status_Update.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending_or_Limited_APIs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field_Fill_Actions'!$A$1:$C$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field_Fill_Actions'!$A$1:$C$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Final_Data_Counts'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pending_or_Limited_APIs'!$A$1:$C$5</definedName>
   </definedNames>
@@ -431,11 +431,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="53" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -541,8 +541,25 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Technology_Detail</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Corrected to real signal rows only</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Removed negative placeholder rows such as No print/MPS/collaboration/UC signal; detail sheet now contains only detected hardware/device/endpoint and print/MPS/UC signals from API technology records.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C6"/>
+  <autoFilter ref="A1:C7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>